<commit_message>
actualizados componentes a 1000 pcbs
</commit_message>
<xml_diff>
--- a/Components/componentes.xlsx
+++ b/Components/componentes.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaest\OneDrive\Documentos\4_TELECO\4_2_TELECO\ELCO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48945CEB-C200-4788-A39C-4A5C2D614B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE3D206-C82B-4083-9DBF-EC3DC9056616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Original" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>Cantidad</t>
   </si>
@@ -137,13 +150,19 @@
   </si>
   <si>
     <t>356-ESP32WRVE26464PC</t>
+  </si>
+  <si>
+    <t>PCB NUM</t>
+  </si>
+  <si>
+    <t>COMPONENTS PER PCB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +178,14 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -201,12 +228,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -509,314 +537,474 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="32.109375" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" customWidth="1"/>
+    <col min="4" max="4" width="21.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>5</v>
+        <f>D2*$C$2</f>
+        <v>1000</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2">
+        <v>1000</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>10</v>
+        <f t="shared" ref="A3:A38" si="0">D3*$C$2</f>
+        <v>2000</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>3000</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>45</v>
+        <f t="shared" si="0"/>
+        <v>9000</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>35</v>
+        <f t="shared" si="0"/>
+        <v>7000</v>
       </c>
       <c r="B8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B13" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B14" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B17" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B19" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B20" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B21" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B22" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B23" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B24" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>6000</v>
       </c>
       <c r="B25" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>40</v>
+        <f t="shared" si="0"/>
+        <v>8000</v>
       </c>
       <c r="B26" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D26">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>3000</v>
       </c>
       <c r="B27" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B28" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>4000</v>
       </c>
       <c r="B29" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B30" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>4000</v>
       </c>
       <c r="B31" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>3000</v>
       </c>
       <c r="B32" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B33" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B34" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B35" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>1000</v>
       </c>
       <c r="B36" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B37" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="2">
-        <v>10</v>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="G37" s="2"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <f t="shared" si="0"/>
+        <v>2000</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>36</v>
+      </c>
+      <c r="D38">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>